<commit_message>
INSERTION is working, need to alter the DB to take the in the practice Data correctly.
</commit_message>
<xml_diff>
--- a/Gym_Database_Dataset.xlsx
+++ b/Gym_Database_Dataset.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="MembershipPlan" sheetId="1" state="visible" r:id="rId3"/>
@@ -253,6 +253,7 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -312,8 +313,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -443,90 +448,90 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.98"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>29.99</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>49.99</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>79.99</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>299.99</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>19.99</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>1</v>
       </c>
     </row>
@@ -549,92 +554,92 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.69"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="23.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="21.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="23.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="21.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>101</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>102</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>103</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>104</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>105</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>5</v>
       </c>
     </row>
@@ -658,68 +663,68 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>201</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>202</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>203</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>204</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>205</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>34</v>
       </c>
     </row>
@@ -741,88 +746,93 @@
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.63"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>301</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>202</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>302</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>303</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>201</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>304</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>204</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>305</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>205</v>
       </c>
     </row>
@@ -846,86 +856,86 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>401</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>402</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>403</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>404</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>405</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>54</v>
       </c>
     </row>
@@ -948,112 +958,112 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="18.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.92"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>501</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="D2" s="0" t="n">
+      <c r="D2" s="1" t="n">
         <v>101</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>201</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>502</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>102</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>202</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>503</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>103</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>203</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>504</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>75</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>104</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>204</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>505</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>105</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>205</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Deleted redundant parts of code
</commit_message>
<xml_diff>
--- a/Gym_Database_Dataset.xlsx
+++ b/Gym_Database_Dataset.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MembershipPlan" sheetId="1" state="visible" r:id="rId3"/>
@@ -747,9 +747,9 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -854,6 +854,9 @@
   </sheetPr>
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.38"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>